<commit_message>
Update test cases (add TC19-TC22, fix typos) and fix prompt_log title
</commit_message>
<xml_diff>
--- a/Testcase.xlsx
+++ b/Testcase.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="165">
   <si>
     <t>BẢNG QUẢN LÝ KIỂM THỬ CHẤT LƯỢNG - BẾP HỒNG NGOẠI SUNHOUSE SHD6011</t>
   </si>
@@ -167,7 +167,7 @@
     <t>1.  Thử các nút điều chỉnh nhiệt độ trên máy</t>
   </si>
   <si>
-    <t>Các nút ấn trơn tru không bị kẹt, điều chỉnh được nhiệt d odoj</t>
+    <t>Các nút ấn trơn tru không bị kẹt, điều chỉnh được nhiệt độ</t>
   </si>
   <si>
     <t>Núm bấm trơn tru, nhiệt độ thay đổi nhạy bén.</t>
@@ -345,7 +345,7 @@
     <t>Thời gian đun sôi 1 lít nước nằm trong khoảng tiêu chuẩn của bếp 2000W (khoảng 3 - 5 phút), chứng tỏ hiệu suất mâm nhiệt tốt.</t>
   </si>
   <si>
-    <t>3 TEST CASES BỔ SUNG</t>
+    <t xml:space="preserve"> TEST CASES TỰ  BỔ SUNG</t>
   </si>
   <si>
     <t>TC16</t>
@@ -406,31 +406,137 @@
     <t>Đế cao su bám dính tốt, bếp vững vàng không bị xê dịch khi tác động lực.</t>
   </si>
   <si>
-    <t>GIẢI THÍCH LÝ DO VÌ SAO AI TRƯỚC ĐÓ BỎ SÓT</t>
-  </si>
-  <si>
-    <t>Hạng mục kiểm thử</t>
-  </si>
-  <si>
-    <t>Phân tích nguyên nhân AI bỏ sót &amp; Tầm quan trọng thực tế</t>
-  </si>
-  <si>
-    <t>1. Đối với TC16 (Sốc nhiệt mặt kính)</t>
-  </si>
-  <si>
-    <t>Lý do AI sót: Đặc thù lớn nhất của bếp hồng ngoại (so với bếp từ) là mặt kính bị nung nóng trực tiếp bởi bóng halogen/mâm nhiệt bên dưới, nhiệt độ bề mặt có thể lên tới 500-600°C. AI trước đó đã test "độ chịu lực" (TC09 - đè nồi 10kg lên) nhưng lại quên mất điểm yếu vật lý chí mạng nhất của kính là "sốc nhiệt". Quá trình nấu nướng thực tế rất dễ rớt nước lạnh hoặc nước canh từ ngoài vào mâm đang đỏ lửa. AI chỉ tư duy theo hướng "nóng tĩnh" mà thiếu tư duy về "biến thiên nhiệt độ đột ngột".</t>
-  </si>
-  <si>
-    <t>2. Đối với TC17 (Tràn nước vào núm cơ học)</t>
-  </si>
-  <si>
-    <t>Lý do AI sót: AI nhìn thấy thông số "Bếp cơ" và chỉ test xem núm vặn có trơn tru không (TC06). Tuy nhiên, nó không nhận ra một rủi ro UX cực lớn của bếp điều khiển cơ (núm xoay) so với bếp cảm ứng: Núm xoay luôn có khe hở vật lý nối trực tiếp vào mạch bên trong thân máy. Trong môi trường bếp, việc trào nước/canh là xảy ra thường xuyên. AI thiếu "bối cảnh thảm họa nhà bếp" (Kitchen Disaster Context) để test khả năng chống nước xâm nhập tại các khe hở cơ học này.</t>
-  </si>
-  <si>
-    <t>3. Đối với TC18 (Độ bám chống trượt do trọng lượng nhẹ)</t>
-  </si>
-  <si>
-    <t>Lý do AI sót: Ở TC04, AI lấy thông số "1.9 kg" trên nhãn để đi test... xem cân lên có đúng 1.9 kg hay không. Đây là tư duy xác minh thông số rất máy móc. Với một QA phần cứng có kinh nghiệm, khi nhìn thấy một chiếc bếp chỉ nặng 1.9 kg (khá nhẹ), họ sẽ nảy ra ngay câu hỏi về tính Động lực học (Kinetic): "Nếu nó nhẹ thế này, khi đặt chảo lên xào nấu đảo mạnh, lực tay đẩy ngang có làm cả chiếc bếp trượt đi trên mặt bàn trơn không?". AI không có cơ thể vật lý, không nấu ăn bao giờ nên không có cảm quan về lực cản ma sát trong quá trình thao tác xào nấu thực tế.</t>
+    <t>TC19</t>
+  </si>
+  <si>
+    <t>Kiểm tra độ chống xước của mặt kính khi vệ sinh cặn cháy khét cứng đầu.</t>
+  </si>
+  <si>
+    <t>- Bếp hồng ngoại dính cặn thức ăn cháy khét.
+- Bối rửa bát bằng cước sắt/nhôm.</t>
+  </si>
+  <si>
+    <t>1. Để lại vết cặn thức ăn (nước mỡ/mực nướng) cháy khét cứng trên mâm nhiệt.
+2. Dùng bối cước sắt/nhôm chà xát để làm sạch.</t>
+  </si>
+  <si>
+    <t>Bề mặt kính có lớp men bảo vệ đủ độ cứng, không bị xước xát sâu hay bong tróc khi có lực cọ rửa vật lý tác động.</t>
+  </si>
+  <si>
+    <t>Kính xước dăm trắng chi chít, mất men bóng vĩnh viễn, dễ bám cặn hơn ở các lần sau.</t>
+  </si>
+  <si>
+    <t>TC20</t>
+  </si>
+  <si>
+    <t>Kiểm tra thiết kế chống kẹt của quạt tản nhiệt đáy trong môi trường đặt bệt (sàn nhà).</t>
+  </si>
+  <si>
+    <t>- Sàn nhà mô phỏng có bụi, tóc, lông thú.
+- Bếp hoạt động liên tục.</t>
+  </si>
+  <si>
+    <t>1. Đặt bếp bệt trực tiếp xuống mặt sàn nhà (mô phỏng thói quen ăn lẩu).
+2. Bật bếp hoạt động từ 1-2 tiếng.
+3. Kiểm tra lồng quạt đáy bếp.</t>
+  </si>
+  <si>
+    <t>Khe hút gió/lưới bảo vệ của quạt được thiết kế để ngăn cản các dị vật lớn (tóc, nilon) lọt vào trục động cơ; quạt hoạt động êm ái.</t>
+  </si>
+  <si>
+    <t>Tóc, lông thú và nilon cuốn vào trục làm quạt kêu lạch cạch/ù ù rất to, quay lờ đờ.</t>
+  </si>
+  <si>
+    <t>TC21</t>
+  </si>
+  <si>
+    <t>Đánh giá ảnh hưởng của nhiệt dư mặt kính đến món ăn sau khi tắt bếp (Hiện tượng Overcooking).</t>
+  </si>
+  <si>
+    <t>- Nồi chứa món ăn (canh/rau) vừa nấu chín tới.</t>
+  </si>
+  <si>
+    <t>1. Nấu nồi thức ăn đến khi vừa chín tới.
+2. Vặn công suất về 0 (tắt bếp) nhưng để nguyên nồi trên vùng nấu.
+3. Quan sát kết cấu món ăn sau 5-10 phút.</t>
+  </si>
+  <si>
+    <t>Nhiệt dư tản nhanh hoặc không truyền quá mạnh, không làm thay đổi kết cấu món ăn. Người dùng không bắt buộc phải bê nồi ra nơi khác ngay.</t>
+  </si>
+  <si>
+    <t>Nồi tiếp tục sôi thêm 5-10 phút làm thức ăn nhũn nát. Ép người dùng phải bê nồi đi chỗ khác.</t>
+  </si>
+  <si>
+    <t>TC22</t>
+  </si>
+  <si>
+    <t>Kiểm tra trải nghiệm xử lý sự cố rơi vãi thức ăn trên mặt kính đang nung nóng.</t>
+  </si>
+  <si>
+    <t>- Vụn thức ăn/nước chấm.
+- Bếp đang hoạt động ở mức nhiệt độ cao.</t>
+  </si>
+  <si>
+    <t>1. Bật bếp ở công suất Max (mặt kính đạt 400-600°C).
+2. Cố tình làm rơi vãi vụn thức ăn trực tiếp xuống mâm nhiệt đỏ rực.
+3. Quan sát hiện tượng và thử lau chùi ngay.</t>
+  </si>
+  <si>
+    <t>Vết bẩn không phát sinh khói độc hại nghiêm trọng hoặc người dùng có thể can thiệp lau/gạt nhanh chóng để tiếp tục việc nấu nướng.</t>
+  </si>
+  <si>
+    <t>Thức ăn bốc khói khét lẹt ngay lập tức. Không thể lau ngay vì kính quá nóng/sợ cháy khăn, làm gián đoạn hoàn toàn bữa ăn.</t>
+  </si>
+  <si>
+    <t>PHÂN TÍCH NGUYÊN NHÂN AI BỎ SÓT TEST CASES</t>
+  </si>
+  <si>
+    <t>Test Case (Bổ sung)</t>
+  </si>
+  <si>
+    <t>Phân tích nguyên nhân &amp; Hạn chế tư duy của AI</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng chịu sốc nhiệt của mặt kính (Thermal Shock Test)</t>
+  </si>
+  <si>
+    <t>Đặc thù lớn nhất của bếp hồng ngoại (so với bếp từ) là mặt kính bị nung nóng trực tiếp bởi bóng halogen/mâm nhiệt bên dưới, nhiệt độ bề mặt có thể lên tới 500-600°C. AI trước đó đã test "độ chịu lực" (TC09 - đè nồi 10kg lên) nhưng lại quên mất điểm yếu vật lý chí mạng nhất của kính là "sốc nhiệt". Quá trình nấu nướng thực tế rất dễ rớt nước lạnh hoặc nước canh từ ngoài vào mâm đang đỏ lửa. AI chỉ tư duy theo hướng "nóng tĩnh" mà thiếu tư duy về "biến thiên nhiệt độ đột ngột".</t>
+  </si>
+  <si>
+    <t>Kiểm tra an toàn chập điện khi nước trào (Spill/Water Ingress Test)</t>
+  </si>
+  <si>
+    <t>AI nhìn thấy thông số "Bếp cơ" và chỉ test xem núm vặn có trơn tru không (TC06). Tuy nhiên, nó không nhận ra một rủi ro UX cực lớn của bếp điều khiển cơ (núm xoay) so với bếp cảm ứng: Núm xoay luôn có khe hở vật lý nối trực tiếp vào mạch bên trong thân máy. Trong môi trường bếp, việc trào nước/canh là xảy ra thường xuyên. AI thiếu "bối cảnh thảm họa nhà bếp" (Kitchen Disaster Context) để test khả năng chống nước xâm nhập tại các khe hở cơ học này.</t>
+  </si>
+  <si>
+    <t>Kiểm tra độ bám và chống trượt khi thao tác (Ma sát chân đế)</t>
+  </si>
+  <si>
+    <t>Ở TC04, AI lấy thông số "1.9 kg" trên nhãn để đi test... xem cân lên có đúng 1.9 kg hay không. Đây là tư duy xác minh thông số rất máy móc. Với một QA phần cứng có kinh nghiệm, khi nhìn thấy một chiếc bếp chỉ nặng 1.9 kg (khá nhẹ), họ sẽ nảy ra ngay câu hỏi về tính Động lực học (Kinetic): "Nếu nó nhẹ thế này, khi đặt chảo lên xào nấu đảo mạnh, lực tay đẩy ngang có làm cả chiếc bếp trượt đi trên mặt bàn trơn không?". AI không có cơ thể vật lý, không nấu ăn bao giờ nên không có cảm quan về lực cản ma sát trong quá trình thao tác xào nấu thực tế.</t>
+  </si>
+  <si>
+    <t>Kiểm tra độ chống xước của mặt kính khi vệ sinh cặn cháy khét cứng đầu</t>
+  </si>
+  <si>
+    <t>AI thường được huấn luyện dựa trên "Hướng dẫn sử dụng" (User Manual) của nhà sản xuất, trong đó luôn ghi rõ: "Chỉ dùng khăn mềm ẩm để lau mặt kính". AI (như ở TC13) đã ngoan ngoãn làm theo sách vở bằng cách lấy khăn ẩm ra lau. Tuy nhiên, AI không hiểu được hành vi cực đoan của người dùng (Extreme User Behavior). Trong thực tế, nước mỡ hay gia vị rớt xuống mặt kính 500°C sẽ hóa than đóng vảy cực kỳ cứng đầu. Lúc này, người dùng sẽ mất kiên nhẫn và dùng bối rửa bát bằng cước sắt chà xát cật lực. AI không phải nai lưng ra dọn dẹp nên không có "cảm quan về độ lười và sự bất lực" của người dùng khi phải đối mặt với vết bẩn cứng đầu, dẫn đến việc bỏ qua bài test ma sát vật lý cường độ cao này.</t>
+  </si>
+  <si>
+    <t>Kiểm tra thiết kế chống kẹt của quạt tản nhiệt đáy trong môi trường đặt bệt (sàn nhà)</t>
+  </si>
+  <si>
+    <t>Ở TC08, AI đã kiểm tra quạt chạy có êm không, nhưng nó đang tưởng tượng chiếc bếp được đặt trong một môi trường... vô trùng, hoặc trên bàn đá hoa cương sạch sẽ chói lóa. AI thiếu hoàn toàn bối cảnh văn hóa và môi trường sống thực tế (Cultural &amp; Environmental Context). Ở Việt Nam và châu Á, bếp hồng ngoại đơn 90% được mua về để... đặt bệt xuống chiếu/sàn nhà ăn lẩu. Dưới sàn nhà luôn đầy rẫy tóc rụng, bụi bông và lông chó mèo. AI không hiểu được đặc thù sử dụng "bình dân" này nên không nhận ra quạt gió gầm bếp sẽ biến thành một chiếc máy hút bụi bất đắc dĩ.</t>
+  </si>
+  <si>
+    <t>Đánh giá ảnh hưởng của nhiệt dư mặt kính đến món ăn sau khi tắt bếp (Hiện tượng Overcooking)</t>
+  </si>
+  <si>
+    <t>AI đã nhận diện được nhiệt dư ở TC10 (cảnh báo đèn chữ H để tránh phỏng tay). Tuy nhiên, AI chỉ tư duy nhiệt dư dưới lăng kính An toàn vật lý (Safety Hazard) mà hoàn toàn mù tịt về Khoa học ẩm thực (Culinary UX). Bếp tắt rồi nhưng nồi tiếp tục sôi sùng sục làm nhũn nát đĩa rau xào. Với AI, "tắt bếp" là kết thúc Test Case; nhưng với người nội trợ, "tắt bếp" món ăn mới hoàn thành một nửa, họ còn phải rảnh tay đi làm việc khác. AI không ăn uống bao giờ nên không biết thế nào là "nhũn nát", cũng không hiểu sự phiền toái khi cứ phải bưng vác cái nồi đang nóng hổi chạy đi tìm chỗ để tạm.</t>
+  </si>
+  <si>
+    <t>Kiểm tra trải nghiệm xử lý sự cố rơi vãi thức ăn trên mặt kính đang nung nóng</t>
+  </si>
+  <si>
+    <t>AI tư duy theo luồng tuyến tính từng bước (Step-by-step): Bước 1 Nấu xong -&gt; Bước 2 Để nguội -&gt; Bước 3 Lau chùi. AI không lường trước được tính hỗn loạn thời gian thực (Real-time Chaos) trong nhà bếp. Thức ăn rơi ra là bốc khói khét lẹt ngay lập tức (ảnh hưởng khứu giác/hô hấp), nhưng nếu lau ngay bằng khăn ướt thì vỡ kính do sốc nhiệt (TC16), còn đợi nguội thì hỏng bữa cơm. AI không có hệ hô hấp để ngửi thấy mùi khét, cũng không có khả năng "đồng cảm" với sự cuống cuồng, tiến thoái lưỡng nan của người đầu bếp trong tình huống này nên không thể sinh ra bài test UX đánh giá mức độ ức chế.</t>
   </si>
 </sst>
 </file>
@@ -440,7 +546,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="22">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -549,9 +655,18 @@
       <name val="Roboto"/>
     </font>
     <font>
-      <b/>
       <sz val="10.0"/>
-      <color rgb="FF1C4875"/>
+      <color rgb="FF000000"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color rgb="FF1E1E1E"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color rgb="FF333333"/>
       <name val="Roboto"/>
     </font>
   </fonts>
@@ -617,7 +732,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="20">
     <border/>
     <border>
       <left style="thin">
@@ -765,6 +880,17 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="FFDFE4EC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDFE4EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDFE4EC"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FFE0E5ED"/>
       </left>
       <top style="thin">
@@ -793,11 +919,41 @@
         <color rgb="FFE0E5ED"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDFE4EC"/>
+      </left>
+      <top style="thin">
+        <color rgb="FFDFE4EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDFE4EC"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FFDFE4EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDFE4EC"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FFDFE4EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDFE4EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDFE4EC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="51">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -883,23 +1039,56 @@
     <xf borderId="8" fillId="10" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="13" fillId="7" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="8" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="8" fillId="10" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="10" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="10" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="8" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="8" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="8" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="13" fillId="8" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="13" fillId="8" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="13" fillId="8" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="8" fontId="19" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="14" fillId="7" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="15" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="12" fillId="8" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="16" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="8" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="8" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="13" fillId="8" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="17" fillId="8" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="12" fillId="10" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="13" fillId="10" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
+    <xf borderId="18" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="19" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1169,25 +1358,25 @@
     </row>
     <row r="6" ht="33.0" customHeight="1">
       <c r="B6" s="12">
-        <f>COUNTA(B9:B23)</f>
-        <v>15</v>
+        <f>COUNTIF(B9:B34, "TC*")</f>
+        <v>22</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="13">
-        <f>COUNTIF(H9:H23, "Pass")</f>
-        <v>12</v>
+        <f>COUNTIF(H9:H34, "Pass")</f>
+        <v>14</v>
       </c>
       <c r="E6" s="14">
-        <f>COUNTIF(H9:H23, "Fail")</f>
-        <v>1</v>
+        <f>COUNTIF(H9:H34, "Fail")</f>
+        <v>5</v>
       </c>
       <c r="F6" s="15">
-        <f>COUNTIF(H9:H23, "Pending") + COUNTIF(H9:H23, "Blocked")</f>
-        <v>2</v>
+        <f>COUNTIF(H9:H34, "Pending") + COUNTIF(H9:H34, "Blocked")</f>
+        <v>3</v>
       </c>
       <c r="G6" s="16">
         <f>IFERROR(D6/B6, 0)</f>
-        <v>0.8</v>
+        <v>0.6363636364</v>
       </c>
       <c r="H6" s="11"/>
     </row>
@@ -1662,84 +1851,401 @@
         <v>20</v>
       </c>
     </row>
+    <row r="31">
+      <c r="B31" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="C31" s="32" t="s">
+        <v>125</v>
+      </c>
+      <c r="D31" s="32" t="s">
+        <v>126</v>
+      </c>
+      <c r="E31" s="32" t="s">
+        <v>127</v>
+      </c>
+      <c r="F31" s="32" t="s">
+        <v>128</v>
+      </c>
+      <c r="G31" s="33" t="s">
+        <v>129</v>
+      </c>
+      <c r="H31" s="34" t="s">
+        <v>100</v>
+      </c>
+    </row>
     <row r="32">
-      <c r="B32" s="22" t="s">
+      <c r="B32" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="C32" s="36" t="s">
+        <v>131</v>
+      </c>
+      <c r="D32" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="E32" s="36" t="s">
+        <v>133</v>
+      </c>
+      <c r="F32" s="36" t="s">
+        <v>134</v>
+      </c>
+      <c r="G32" s="37" t="s">
+        <v>135</v>
+      </c>
+      <c r="H32" s="38" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="31" t="s">
+        <v>136</v>
+      </c>
+      <c r="C33" s="32" t="s">
+        <v>137</v>
+      </c>
+      <c r="D33" s="32" t="s">
+        <v>138</v>
+      </c>
+      <c r="E33" s="32" t="s">
+        <v>139</v>
+      </c>
+      <c r="F33" s="32" t="s">
+        <v>140</v>
+      </c>
+      <c r="G33" s="33" t="s">
+        <v>141</v>
+      </c>
+      <c r="H33" s="34" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="35" t="s">
+        <v>142</v>
+      </c>
+      <c r="C34" s="39" t="s">
+        <v>143</v>
+      </c>
+      <c r="D34" s="39" t="s">
+        <v>144</v>
+      </c>
+      <c r="E34" s="39" t="s">
+        <v>145</v>
+      </c>
+      <c r="F34" s="39" t="s">
+        <v>146</v>
+      </c>
+      <c r="G34" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="H34" s="41" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="42"/>
+      <c r="C35" s="42"/>
+      <c r="D35" s="42"/>
+      <c r="E35" s="42"/>
+      <c r="F35" s="42"/>
+      <c r="G35" s="42"/>
+      <c r="H35" s="42"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="42"/>
+      <c r="C36" s="42"/>
+      <c r="D36" s="42"/>
+      <c r="E36" s="42"/>
+      <c r="F36" s="42"/>
+      <c r="G36" s="42"/>
+      <c r="H36" s="42"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="C37" s="23"/>
+      <c r="D37" s="23"/>
+      <c r="E37" s="23"/>
+      <c r="F37" s="23"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="24"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="C38" s="25" t="s">
+        <v>149</v>
+      </c>
+      <c r="D38" s="43" t="s">
+        <v>150</v>
+      </c>
+      <c r="E38" s="44"/>
+      <c r="F38" s="44"/>
+      <c r="G38" s="44"/>
+      <c r="H38" s="45"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="46" t="s">
+        <v>107</v>
+      </c>
+      <c r="C39" s="47" t="s">
+        <v>151</v>
+      </c>
+      <c r="D39" s="48" t="s">
+        <v>152</v>
+      </c>
+      <c r="E39" s="49"/>
+      <c r="F39" s="49"/>
+      <c r="G39" s="49"/>
+      <c r="H39" s="50"/>
+    </row>
+    <row r="40">
+      <c r="B40" s="46" t="s">
+        <v>112</v>
+      </c>
+      <c r="C40" s="47" t="s">
+        <v>153</v>
+      </c>
+      <c r="D40" s="48" t="s">
+        <v>154</v>
+      </c>
+      <c r="E40" s="49"/>
+      <c r="F40" s="49"/>
+      <c r="G40" s="49"/>
+      <c r="H40" s="50"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="46" t="s">
+        <v>118</v>
+      </c>
+      <c r="C41" s="47" t="s">
+        <v>155</v>
+      </c>
+      <c r="D41" s="48" t="s">
+        <v>156</v>
+      </c>
+      <c r="E41" s="49"/>
+      <c r="F41" s="49"/>
+      <c r="G41" s="49"/>
+      <c r="H41" s="50"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="46" t="s">
         <v>124</v>
       </c>
-      <c r="C32" s="23"/>
-      <c r="D32" s="23"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="24"/>
-    </row>
-    <row r="33">
-      <c r="B33" s="25" t="s">
-        <v>125</v>
-      </c>
-      <c r="C33" s="31" t="s">
-        <v>126</v>
-      </c>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="33"/>
-    </row>
-    <row r="34">
-      <c r="B34" s="34" t="s">
-        <v>127</v>
-      </c>
-      <c r="C34" s="35" t="s">
-        <v>128</v>
-      </c>
-      <c r="D34" s="32"/>
-      <c r="E34" s="32"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="32"/>
-      <c r="H34" s="33"/>
-    </row>
-    <row r="35">
-      <c r="B35" s="36" t="s">
-        <v>129</v>
-      </c>
-      <c r="C35" s="37" t="s">
+      <c r="C42" s="47" t="s">
+        <v>157</v>
+      </c>
+      <c r="D42" s="48" t="s">
+        <v>158</v>
+      </c>
+      <c r="E42" s="49"/>
+      <c r="F42" s="49"/>
+      <c r="G42" s="49"/>
+      <c r="H42" s="50"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="46" t="s">
         <v>130</v>
       </c>
-      <c r="D35" s="32"/>
-      <c r="E35" s="32"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
-      <c r="H35" s="33"/>
-    </row>
-    <row r="36">
-      <c r="B36" s="34" t="s">
-        <v>131</v>
-      </c>
-      <c r="C36" s="35" t="s">
-        <v>132</v>
-      </c>
-      <c r="D36" s="32"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
-      <c r="H36" s="33"/>
+      <c r="C43" s="47" t="s">
+        <v>159</v>
+      </c>
+      <c r="D43" s="48" t="s">
+        <v>160</v>
+      </c>
+      <c r="E43" s="49"/>
+      <c r="F43" s="49"/>
+      <c r="G43" s="49"/>
+      <c r="H43" s="50"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="46" t="s">
+        <v>136</v>
+      </c>
+      <c r="C44" s="47" t="s">
+        <v>161</v>
+      </c>
+      <c r="D44" s="48" t="s">
+        <v>162</v>
+      </c>
+      <c r="E44" s="49"/>
+      <c r="F44" s="49"/>
+      <c r="G44" s="49"/>
+      <c r="H44" s="50"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="46" t="s">
+        <v>142</v>
+      </c>
+      <c r="C45" s="47" t="s">
+        <v>163</v>
+      </c>
+      <c r="D45" s="48" t="s">
+        <v>164</v>
+      </c>
+      <c r="E45" s="49"/>
+      <c r="F45" s="49"/>
+      <c r="G45" s="49"/>
+      <c r="H45" s="50"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="42"/>
+      <c r="C46" s="42"/>
+      <c r="D46" s="42"/>
+      <c r="E46" s="42"/>
+      <c r="F46" s="42"/>
+      <c r="G46" s="42"/>
+      <c r="H46" s="42"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="42"/>
+      <c r="C47" s="42"/>
+      <c r="D47" s="42"/>
+      <c r="E47" s="42"/>
+      <c r="F47" s="42"/>
+      <c r="G47" s="42"/>
+      <c r="H47" s="42"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="42"/>
+      <c r="C48" s="42"/>
+      <c r="D48" s="42"/>
+      <c r="E48" s="42"/>
+      <c r="F48" s="42"/>
+      <c r="G48" s="42"/>
+      <c r="H48" s="42"/>
+    </row>
+    <row r="49">
+      <c r="B49" s="42"/>
+      <c r="C49" s="42"/>
+      <c r="D49" s="42"/>
+      <c r="E49" s="42"/>
+      <c r="F49" s="42"/>
+      <c r="G49" s="42"/>
+      <c r="H49" s="42"/>
+    </row>
+    <row r="50">
+      <c r="B50" s="42"/>
+      <c r="C50" s="42"/>
+      <c r="D50" s="42"/>
+      <c r="E50" s="42"/>
+      <c r="F50" s="42"/>
+      <c r="G50" s="42"/>
+      <c r="H50" s="42"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="42"/>
+      <c r="C51" s="42"/>
+      <c r="D51" s="42"/>
+      <c r="E51" s="42"/>
+      <c r="F51" s="42"/>
+      <c r="G51" s="42"/>
+      <c r="H51" s="42"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="42"/>
+      <c r="C52" s="42"/>
+      <c r="D52" s="42"/>
+      <c r="E52" s="42"/>
+      <c r="F52" s="42"/>
+      <c r="G52" s="42"/>
+      <c r="H52" s="42"/>
+    </row>
+    <row r="53">
+      <c r="B53" s="42"/>
+      <c r="C53" s="42"/>
+      <c r="D53" s="42"/>
+      <c r="E53" s="42"/>
+      <c r="F53" s="42"/>
+      <c r="G53" s="42"/>
+      <c r="H53" s="42"/>
+    </row>
+    <row r="54">
+      <c r="B54" s="42"/>
+      <c r="C54" s="42"/>
+      <c r="D54" s="42"/>
+      <c r="E54" s="42"/>
+      <c r="F54" s="42"/>
+      <c r="G54" s="42"/>
+      <c r="H54" s="42"/>
+    </row>
+    <row r="55">
+      <c r="B55" s="42"/>
+      <c r="C55" s="42"/>
+      <c r="D55" s="42"/>
+      <c r="E55" s="42"/>
+      <c r="F55" s="42"/>
+      <c r="G55" s="42"/>
+      <c r="H55" s="42"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="42"/>
+      <c r="C56" s="42"/>
+      <c r="D56" s="42"/>
+      <c r="E56" s="42"/>
+      <c r="F56" s="42"/>
+      <c r="G56" s="42"/>
+      <c r="H56" s="42"/>
+    </row>
+    <row r="57">
+      <c r="B57" s="42"/>
+      <c r="C57" s="42"/>
+      <c r="D57" s="42"/>
+      <c r="E57" s="42"/>
+      <c r="F57" s="42"/>
+      <c r="G57" s="42"/>
+      <c r="H57" s="42"/>
+    </row>
+    <row r="58">
+      <c r="B58" s="42"/>
+      <c r="C58" s="42"/>
+      <c r="D58" s="42"/>
+      <c r="E58" s="42"/>
+      <c r="F58" s="42"/>
+      <c r="G58" s="42"/>
+      <c r="H58" s="42"/>
+    </row>
+    <row r="59">
+      <c r="B59" s="42"/>
+      <c r="C59" s="42"/>
+      <c r="D59" s="42"/>
+      <c r="E59" s="42"/>
+      <c r="F59" s="42"/>
+      <c r="G59" s="42"/>
+      <c r="H59" s="42"/>
+    </row>
+    <row r="60">
+      <c r="B60" s="42"/>
+      <c r="C60" s="42"/>
+      <c r="D60" s="42"/>
+      <c r="E60" s="42"/>
+      <c r="F60" s="42"/>
+      <c r="G60" s="42"/>
+      <c r="H60" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="C36:H36"/>
+  <mergeCells count="14">
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="D40:H40"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="D45:H45"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="B26:H26"/>
-    <mergeCell ref="B32:H32"/>
-    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="D38:H38"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="H9:H23 H28:H30">
+    <dataValidation type="list" allowBlank="1" sqref="H9:H23 H28:H34">
       <formula1>"Pending,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>